<commit_message>
Add 3 Instagram-sourced wedding vendor leads
Loviebeks Photography, Nell's Florals, Charleston Bride Tribe -
all active, all lacking a real website (CRM intake form,
no link, or Linktree only). Confirmed via IG follower/post counts.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N63pwWHxLLsDgQhVNkSpwX
</commit_message>
<xml_diff>
--- a/lead-tracker.xlsx
+++ b/lead-tracker.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="130">
   <si>
     <t xml:space="preserve">Business Name</t>
   </si>
@@ -333,6 +333,36 @@
   </si>
   <si>
     <t xml:space="preserve">Event management company, 4.4 stars (20 reviews). No website on Maps, likely home-based.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loviebeks Photography</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@loviebeks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charleston, SC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IG: Charleston Wedding Photographer, 5114 followers, 1301 posts (very active). Bio link is a Dubsado CRM intake form, not a real site. Confirm actual business/brand name on first contact.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nell's Florals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@nellsflorals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IG: Charleston Wedding Florist, owner Jenn Sexton, 411 followers. No bio link at all.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charleston Bride Tribe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@charlestonbridetribe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IG: #1 Charleston Bachelorette Photographer, 3252 followers, 175 posts (very active). Bio link is only a Linktree, no real website.</t>
   </si>
   <si>
     <t xml:space="preserve">Legend / Instructions</t>
@@ -1547,48 +1577,96 @@
       <c r="M15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
+      <c r="A16" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>105</v>
+      </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
+      <c r="F16" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="I16" s="7"/>
       <c r="J16" s="7"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="8"/>
+      <c r="K16" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="L16" s="8" t="n">
+        <v>46288</v>
+      </c>
       <c r="M16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
+      <c r="A17" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>109</v>
+      </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
+      <c r="F17" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="I17" s="7"/>
       <c r="J17" s="7"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="8"/>
+      <c r="K17" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="L17" s="8" t="n">
+        <v>46288</v>
+      </c>
       <c r="M17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
+      <c r="A18" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>112</v>
+      </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
+      <c r="F18" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="I18" s="7"/>
       <c r="J18" s="7"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="8"/>
+      <c r="K18" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="L18" s="8" t="n">
+        <v>46288</v>
+      </c>
       <c r="M18" s="8"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2088,27 +2166,27 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="10" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="10" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="10" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="10" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -2179,30 +2257,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="B4" s="13" t="n">
         <f aca="false">COUNTA(Leads!A2:A51)</f>
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2220,7 +2298,7 @@
       </c>
       <c r="B8" s="15" t="n">
         <f aca="false">COUNTIF(Leads!H2:H51,A8)</f>
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2297,7 +2375,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="B18" s="13" t="n">
         <f aca="false">COUNTIF(Leads!H2:H51,"DM Sent")+COUNTIF(Leads!H2:H51,"Replied")+COUNTIF(Leads!H2:H51,"WhatsApp")+COUNTIF(Leads!H2:H51,"Demo Sent")+COUNTIF(Leads!H2:H51,"Negotiating")+COUNTIF(Leads!H2:H51,"Deposit Paid")+COUNTIF(Leads!H2:H51,"Won")+COUNTIF(Leads!H2:H51,"Lost/Ghosted")</f>
@@ -2306,7 +2384,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="B20" s="13" t="n">
         <f aca="false">COUNTIF(Leads!H2:H51,"Won")</f>
@@ -2315,7 +2393,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="B21" s="22" t="n">
         <f aca="false">IFERROR(B20/B18,0)</f>
@@ -2324,7 +2402,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="B23" s="23" t="n">
         <f aca="false">SUM(Leads!J2:J51)</f>
@@ -2333,7 +2411,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="B24" s="23" t="n">
         <f aca="false">SUMIF(Leads!H2:H51,"Won",Leads!I2:I51)+SUMIF(Leads!H2:H51,"Deposit Paid",Leads!I2:I51)</f>
@@ -2342,7 +2420,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B25" s="23" t="n">
         <f aca="false">IFERROR(SUMIF(Leads!H2:H51,"Won",Leads!I2:I51)/B20,0)</f>
@@ -2351,7 +2429,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12"/>

</xml_diff>

<commit_message>
Add Rachel Craig Photography lead
Wedding photographer, 5.0 stars (16 reviews), no website on Maps.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N63pwWHxLLsDgQhVNkSpwX
</commit_message>
<xml_diff>
--- a/lead-tracker.xlsx
+++ b/lead-tracker.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="134">
   <si>
     <t xml:space="preserve">Business Name</t>
   </si>
@@ -363,6 +363,18 @@
   </si>
   <si>
     <t xml:space="preserve">IG: #1 Charleston Bachelorette Photographer, 3252 followers, 175 posts (very active). Bio link is only a Linktree, no real website.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rachel Craig Photography</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://google.com/maps/place/Rachel+Craig+Photography</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+1 843-743-8567</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wedding photographer, 5.0 stars (16 reviews), listing shows Open. No website (Maps flags it as missing info). Search IG for handle before outreach.</t>
   </si>
   <si>
     <t xml:space="preserve">Legend / Instructions</t>
@@ -1670,18 +1682,36 @@
       <c r="M18" s="8"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6"/>
-      <c r="B19" s="6"/>
+      <c r="A19" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>14</v>
+      </c>
       <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
+      <c r="D19" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="I19" s="7"/>
       <c r="J19" s="7"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="8"/>
+      <c r="K19" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="L19" s="8" t="n">
+        <v>46288</v>
+      </c>
       <c r="M19" s="8"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2166,27 +2196,27 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="10" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="10" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="10" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="10" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -2257,30 +2287,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B4" s="13" t="n">
         <f aca="false">COUNTA(Leads!A2:A51)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2298,7 +2328,7 @@
       </c>
       <c r="B8" s="15" t="n">
         <f aca="false">COUNTIF(Leads!H2:H51,A8)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2375,7 +2405,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B18" s="13" t="n">
         <f aca="false">COUNTIF(Leads!H2:H51,"DM Sent")+COUNTIF(Leads!H2:H51,"Replied")+COUNTIF(Leads!H2:H51,"WhatsApp")+COUNTIF(Leads!H2:H51,"Demo Sent")+COUNTIF(Leads!H2:H51,"Negotiating")+COUNTIF(Leads!H2:H51,"Deposit Paid")+COUNTIF(Leads!H2:H51,"Won")+COUNTIF(Leads!H2:H51,"Lost/Ghosted")</f>
@@ -2384,7 +2414,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B20" s="13" t="n">
         <f aca="false">COUNTIF(Leads!H2:H51,"Won")</f>
@@ -2393,7 +2423,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B21" s="22" t="n">
         <f aca="false">IFERROR(B20/B18,0)</f>
@@ -2402,7 +2432,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B23" s="23" t="n">
         <f aca="false">SUM(Leads!J2:J51)</f>
@@ -2411,7 +2441,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B24" s="23" t="n">
         <f aca="false">SUMIF(Leads!H2:H51,"Won",Leads!I2:I51)+SUMIF(Leads!H2:H51,"Deposit Paid",Leads!I2:I51)</f>
@@ -2420,7 +2450,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B25" s="23" t="n">
         <f aca="false">IFERROR(SUMIF(Leads!H2:H51,"Won",Leads!I2:I51)/B20,0)</f>
@@ -2429,7 +2459,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12"/>

</xml_diff>